<commit_message>
Fix load tests (Locust & k6) to bypass rate limit with pre-generated token and correct API endpoints
</commit_message>
<xml_diff>
--- a/load-tests/results/Load_Test_Report.xlsx
+++ b/load-tests/results/Load_Test_Report.xlsx
@@ -124,10 +124,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -523,7 +523,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-08 15:37:24</t>
+          <t>2026-08-08 20:26:47</t>
         </is>
       </c>
     </row>
@@ -607,67 +607,127 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Run Locust first to generate CSV data</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Requests / Second</t>
+          <t>Total Failures</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Avg Response Time</t>
+          <t>Requests / Second</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>119.17024426140544</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Min Response Time</t>
+          <t>Avg Response Time</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>52.19043999677524 ms</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Max Response Time</t>
+          <t>Min Response Time</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>42.08749998360872 ms</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Max Response Time</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>79.18570004403591 ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Median Response Time</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>49 ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>90th Percentile</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>79 ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>95th Percentile</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>79 ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>99th Percentile</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>79 ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>Failure Rate</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>0.0 %</t>
         </is>
       </c>
     </row>
@@ -685,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -771,9 +831,124 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>No data yet — run Locust first to populate this sheet.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>[Setup] Session Check</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>52.19043999677524</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>42.08749998360872</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>79.18570004403591</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>119.17024426140544</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr"/>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Aggregated</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>52.19043999677524</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>42.08749998360872</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>79.18570004403591</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>119.17024426140544</t>
         </is>
       </c>
     </row>
@@ -797,7 +972,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Response Time Benchmark Guide</t>
         </is>
@@ -826,34 +1001,34 @@
       <c r="C3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>&lt; 100 ms</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Instant — feels instantaneous</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Excellent</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>100-300 ms</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Fast — user notices no lag</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Good</t>
         </is>

</xml_diff>